<commit_message>
Agregar opcion listar empleados
</commit_message>
<xml_diff>
--- a/ExcelJava/empleados.xlsx
+++ b/ExcelJava/empleados.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>ID</t>
   </si>
@@ -36,6 +36,12 @@
   </si>
   <si>
     <t>Liliana</t>
+  </si>
+  <si>
+    <t>manolo</t>
+  </si>
+  <si>
+    <t>piter</t>
   </si>
 </sst>
 </file>
@@ -80,7 +86,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -93,49 +99,41 @@
     </row>
     <row r="2">
       <c r="A2" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n" s="0">
-        <v>3.0</v>
+        <v>5.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n" s="0">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n" s="0">
-        <v>6.0</v>
-      </c>
-      <c r="B7" t="s" s="0">
         <v>7</v>
       </c>
     </row>

</xml_diff>